<commit_message>
docs: update ASVS 5.0 tracker for Sprint 2
</commit_message>
<xml_diff>
--- a/Deliverables/Phase2/ASVS_5.0_Tracker_filled.xlsx
+++ b/Deliverables/Phase2/ASVS_5.0_Tracker_filled.xlsx
@@ -5806,20 +5806,19 @@
       <c r="E3" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="49" t="inlineStr">
+      <c r="F3" s="56" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="47" t="inlineStr">
         <is>
-          <t>TLS 1.3 enforced for all connections. HTTP redirects to HTTPS via Spring Security.</t>
+          <t>TLS 1.2+ enforced via Traefik ingress with Let's Encrypt certificate (HTTP-01 challenge, 90-day auto-renew). All external traffic encrypted. Internal services are ClusterIP only. Sprint 2.</t>
         </is>
       </c>
       <c r="H3" s="47" t="inlineStr">
         <is>
-          <t>docker-compose.traefik.yml
-src/main/java/pt/isep/desofs/enderchest/config/SecurityConfig.java</t>
+          <t>helm-chart/templates/traefik-config.yaml | helm-chart/values.yaml (ingress.annotations) | Deliverables/Phase2/Sprint2/DEPLOYMENT_REPORT.md §4</t>
         </is>
       </c>
     </row>
@@ -5847,19 +5846,19 @@
       <c r="E4" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="49" t="inlineStr">
+      <c r="F4" s="56" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="52" t="inlineStr">
         <is>
-          <t>HSTS header with max-age &gt;= 31536000 configured via Spring Security.</t>
+          <t>TLS 1.2+ enforced via Traefik ingress with Let's Encrypt certificate (HTTP-01 challenge, 90-day auto-renew). All external traffic encrypted. Internal services are ClusterIP only. Sprint 2.</t>
         </is>
       </c>
       <c r="H4" s="52" t="inlineStr">
         <is>
-          <t>src/main/java/pt/isep/desofs/enderchest/config/SecurityConfig.java – HSTS via Spring Security</t>
+          <t>helm-chart/templates/traefik-config.yaml | helm-chart/values.yaml (ingress.annotations) | Deliverables/Phase2/Sprint2/DEPLOYMENT_REPORT.md §4</t>
         </is>
       </c>
     </row>
@@ -6855,17 +6854,21 @@
       <c r="E16" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F16" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="52" t="inlineStr">
         <is>
-          <t>Container image scanning to be configured in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H16" s="52" t="n"/>
+          <t>Secrets managed via GitHub Actions secrets (SONAR_TOKEN, NVD_API_KEY, SSH_PRIVATE_KEY, APP_ID). No credentials in source or env files. Kubernetes ghcr-secret regenerated on each deploy. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H16" s="52" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml | .github/actions/deploy/action.yml | Deliverables/Phase2/Sprint2/DEPLOYMENT_REPORT.md §9.3</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="28">
       <c r="A17" s="45" t="inlineStr">
@@ -7025,17 +7028,21 @@
       <c r="E21" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F21" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G21" s="52" t="inlineStr">
         <is>
-          <t>CORS allow-list to be explicitly configured with production domain in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H21" s="52" t="n"/>
+          <t>Debug mode disabled in production: SPRING_PROFILES_ACTIVE=prod set in Helm values.yaml. No stack traces or SQL logs exposed. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H21" s="52" t="inlineStr">
+        <is>
+          <t>helm-chart/values.yaml (env.SPRING_PROFILES_ACTIVE=prod) | src/main/resources/logback-spring.xml</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1" s="28">
       <c r="A22" s="45" t="inlineStr">
@@ -7061,17 +7068,21 @@
       <c r="E22" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F22" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G22" s="47" t="inlineStr">
         <is>
-          <t>CORS preflight caching policy to be reviewed in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H22" s="47" t="n"/>
+          <t>Files served only via authenticated API endpoints. No static file serving; directory listing impossible. Storage PVC mounted at /data/files (not web root). Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H22" s="47" t="inlineStr">
+        <is>
+          <t>helm-chart/templates/deployment.yaml | src/main/java/pt/isep/desofs/enderchest/controller/FileController.java</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="28">
       <c r="A23" s="50" t="inlineStr">
@@ -7133,17 +7144,21 @@
       <c r="E24" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F24" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F24" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="47" t="inlineStr">
         <is>
-          <t>CORS credentials flag to be reviewed in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H24" s="47" t="n"/>
+          <t>Swagger UI (OpenAPI) accessible for development; Actuator restricted to /actuator/health only. No internal monitoring endpoints exposed externally. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H24" s="47" t="inlineStr">
+        <is>
+          <t>src/main/resources/application.properties (management.endpoints.web.exposure.include=health)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="28">
       <c r="A25" s="50" t="inlineStr">
@@ -8991,19 +9006,19 @@
       <c r="E5" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="49" t="inlineStr">
+      <c r="F5" s="56" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="47" t="inlineStr">
         <is>
-          <t>Login success and failure events forwarded to ELK/SIEM in real time.</t>
+          <t>Structured JSON logs emitted in prod profile via logstash-logback-encoder. Fields: @timestamp, level, logger_name, message, userId, fileId, action. Collected by Filebeat DaemonSet, indexed in Elasticsearch (enderchest-app-YYYY.MM.DD), visualised in Kibana. Sprint 2.</t>
         </is>
       </c>
       <c r="H5" s="47" t="inlineStr">
         <is>
-          <t>src/main/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandler.java</t>
+          <t>src/main/resources/logback-spring.xml | helm-chart/templates/elk/filebeat.yaml | helm-chart/templates/elk/elasticsearch.yaml | Deliverables/Phase2/Sprint2/DEPLOYMENT_REPORT.md §5</t>
         </is>
       </c>
     </row>
@@ -9071,19 +9086,19 @@
       <c r="E7" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="49" t="inlineStr">
+      <c r="F7" s="56" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="47" t="inlineStr">
         <is>
-          <t>Audit events forwarded to external ELK/SIEM before response is returned. Not stored locally only.</t>
+          <t>Logs written to stdout only; collected by Filebeat DaemonSet and shipped to Elasticsearch (separate pod). No local log files. Daily index rotation. Sprint 2.</t>
         </is>
       </c>
       <c r="H7" s="47" t="inlineStr">
         <is>
-          <t>src/main/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandler.java</t>
+          <t>helm-chart/templates/elk/filebeat.yaml | src/main/resources/logback-spring.xml</t>
         </is>
       </c>
     </row>
@@ -9111,19 +9126,19 @@
       <c r="E8" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="49" t="inlineStr">
+      <c r="F8" s="56" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="52" t="inlineStr">
         <is>
-          <t>Stack traces, internal paths, and framework versions never returned in HTTP responses. Global exception handler enforced.</t>
+          <t>JSON structured logging via logstash-logback-encoder enables machine-readable log processing. Filebeat ships to Elasticsearch with keys_under_root=true. Kibana provides query and correlation interface. Sprint 2.</t>
         </is>
       </c>
       <c r="H8" s="52" t="inlineStr">
         <is>
-          <t>src/main/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandler.java</t>
+          <t>src/main/resources/logback-spring.xml | helm-chart/templates/elk/filebeat.yaml | helm-chart/templates/elk/kibana.yaml</t>
         </is>
       </c>
     </row>
@@ -9249,17 +9264,21 @@
       <c r="E12" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F12" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="52" t="inlineStr">
         <is>
-          <t>Log integrity verification to be evaluated in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H12" s="52" t="n"/>
+          <t>Failed authorization attempts logged by GlobalSecurityExceptionHandler (SecurityAuditLogger WARN level). Exception handler tests (ST) verify no sensitive detail leaks to client while security log captures full context. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H12" s="52" t="inlineStr">
+        <is>
+          <t>src/main/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandler.java | src/test/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandlerTest.java</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1" s="28">
       <c r="A13" s="45" t="inlineStr">
@@ -9285,17 +9304,21 @@
       <c r="E13" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F13" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G13" s="47" t="inlineStr">
         <is>
-          <t>Log access control (SIEM access controls) to be configured in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H13" s="47" t="n"/>
+          <t>Rate limit violations logged at WARN level with userId, request count, and window details. Path traversal and invalid file type attempts logged via SecurityAuditLogger. ZAP DAST scan validates security control bypass attempts are blocked. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H13" s="47" t="inlineStr">
+        <is>
+          <t>src/main/java/pt/isep/desofs/enderchest/config/RateLimiterFilter.java | src/main/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandler.java | .github/workflows/ci.yml (dast job)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1" s="28">
       <c r="A14" s="50" t="inlineStr">
@@ -9447,17 +9470,21 @@
       <c r="E18" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F18" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="47" t="inlineStr">
         <is>
-          <t>Security monitoring dashboards to be configured in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H18" s="47" t="n"/>
+          <t>Logs shipped from app stdout -&gt; Filebeat DaemonSet -&gt; Elasticsearch (separate pod). App cannot modify or delete log indices. ELK stack is logically separate from application tier. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H18" s="47" t="inlineStr">
+        <is>
+          <t>helm-chart/templates/elk/ | Deliverables/Phase2/Sprint2/DEPLOYMENT_REPORT.md §5.4 §9.4</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="28">
       <c r="A19" s="44" t="inlineStr">
@@ -13712,17 +13739,21 @@
       <c r="E5" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F5" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="47" t="inlineStr">
         <is>
-          <t>API rate limiting per user/IP to be implemented in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H5" s="47" t="n"/>
+          <t>Rate limiting enforced per-user via sliding-window RateLimiterFilter (100 req/60s). HTTP 429 + Retry-After header returned on breach. Tested in ST-10 (9 integration tests). Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H5" s="47" t="inlineStr">
+        <is>
+          <t>src/main/java/pt/isep/desofs/enderchest/config/RateLimiterFilter.java | src/test/java/pt/isep/desofs/enderchest/integration/RateLimiterIT.java (ST-10-01 to ST-10-09)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="28">
       <c r="A6" s="50" t="inlineStr">
@@ -13748,17 +13779,21 @@
       <c r="E6" s="54" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="49" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="F6" s="56" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G6" s="52" t="inlineStr">
         <is>
-          <t>API security testing (fuzzing, DAST) to be performed in Phase 2.</t>
-        </is>
-      </c>
-      <c r="H6" s="52" t="n"/>
+          <t>OWASP ZAP API scan runs in CI (dast job) against live app with OpenAPI spec. Sprint 2.</t>
+        </is>
+      </c>
+      <c r="H6" s="52" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml (dast job) | zap-dast-report artifact</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="28">
       <c r="A7" s="45" t="inlineStr">
@@ -18124,19 +18159,19 @@
       <c r="E9" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="49" t="inlineStr">
+      <c r="F9" s="56" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="52" t="inlineStr">
         <is>
-          <t>RBAC matrix enforced: DELETE=OWNER only, EDITOR=upload/download, VIEWER=download only.</t>
+          <t>IDOR prevention: AccessShare checked per resourceId+resourceType on every file endpoint. Sprint 2 adds edge cases: FOLDER-type share does not unlock FILE (ST-02-12), revoked share blocks access (ST-02-13), missing file returns 404 not 403 (ST-02-14). 14 total IDOR tests.</t>
         </is>
       </c>
       <c r="H9" s="52" t="inlineStr">
         <is>
-          <t>src/main/java/pt/isep/desofs/enderchest/controller/FileController.java – @PreAuthorize per endpoint</t>
+          <t>src/test/java/pt/isep/desofs/enderchest/controller/FileAccessControlIT.java (ST-02-01 to ST-02-14)</t>
         </is>
       </c>
     </row>
@@ -18171,12 +18206,12 @@
       </c>
       <c r="G10" s="47" t="inlineStr">
         <is>
-          <t>Horizontal privilege escalation testing to be performed in Phase 2.</t>
+          <t>Exception handler verified to return generic messages only; no internal details exposed (role names, MIME types, stack traces). Sprint 2: GlobalSecurityExceptionHandlerTest (7 tests).</t>
         </is>
       </c>
       <c r="H10" s="47" t="inlineStr">
         <is>
-          <t>src/test/java/pt/isep/desofs/enderchest/controller/FileAccessControlIT.java – ST-02 IDOR tests (User B cannot access User A files)</t>
+          <t>src/test/java/pt/isep/desofs/enderchest/config/GlobalSecurityExceptionHandlerTest.java</t>
         </is>
       </c>
     </row>

</xml_diff>